<commit_message>
Per-row billing currency, PDF without VAT column and Amount last, paste-safe email, no-liability-in-transit term
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJvBMaWnTbAZB6PnjuNkNU
</commit_message>
<xml_diff>
--- a/tools/Sasco_Quote_Templates_v3.xlsx
+++ b/tools/Sasco_Quote_Templates_v3.xlsx
@@ -1563,7 +1563,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
@@ -2791,7 +2790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5609,6 +5608,48 @@
       <c r="H67" s="14" t="inlineStr">
         <is>
           <t>Based on app's Incoterm descriptions - confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>T068</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E68" s="14" t="inlineStr">
+        <is>
+          <t>SASCO Global shall not be responsible or liable for any loss of, or damage to, cargo while in transit, whether by sea, air or land. Cargo insurance is the customer's responsibility.</t>
+        </is>
+      </c>
+      <c r="F68" s="14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G68" s="14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H68" s="14" t="inlineStr">
+        <is>
+          <t>Added by Claude per Nikhil 21-Oct</t>
         </is>
       </c>
     </row>

</xml_diff>